<commit_message>
Removed old parameter set
</commit_message>
<xml_diff>
--- a/publication_simulations/params_SRSF6_Multi_Cell_Hyp/parameters_2.xlsx
+++ b/publication_simulations/params_SRSF6_Multi_Cell_Hyp/parameters_2.xlsx
@@ -388,7 +388,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="0" t="n">
-        <v>3050000</v>
+        <v>4190000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -396,7 +396,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="0" t="n">
-        <v>2200000</v>
+        <v>3020000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -404,7 +404,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="0" t="n">
-        <v>1200000</v>
+        <v>1710000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -468,7 +468,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="0" t="n">
-        <v>1620000</v>
+        <v>2220000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>